<commit_message>
docs: user onboarding — full process docs, improved Excel export, expanded improvement plan with commit links
</commit_message>
<xml_diff>
--- a/docs/user-feedback.xlsx
+++ b/docs/user-feedback.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -33,14 +33,28 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="00888888"/>
+      <i val="1"/>
+      <color rgb="00555555"/>
     </font>
     <font>
       <i val="1"/>
-      <color rgb="00888888"/>
+      <color rgb="00777777"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -49,17 +63,32 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001E3A5F"/>
+        <fgColor rgb="001A1A2E"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F0F4FA"/>
+        <fgColor rgb="00F0F4FF"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFFFFF"/>
+        <fgColor rgb="00FAFAFA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="000F3460"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F5F5F5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E8F4FD"/>
       </patternFill>
     </fill>
   </fills>
@@ -89,20 +118,40 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -468,19 +517,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:G32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
     <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="58" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
     <col width="45" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1">
+    <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>#</t>
@@ -503,7 +552,7 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Product Rating (1–5)</t>
+          <t>Product Rating (1–5 ★)</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
@@ -521,35 +570,35 @@
       <c r="A2" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="inlineStr"/>
-      <c r="C2" s="2" t="inlineStr"/>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="B2" s="3" t="n"/>
+      <c r="C2" s="3" t="n"/>
+      <c r="D2" s="3" t="inlineStr">
         <is>
           <t>GC4COEPJQRXZFTRZJYOYEIHVX6OCSZD5GMOAI6JGRDM3Y33VKBLODYUE</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr"/>
-      <c r="F2" s="2" t="inlineStr"/>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="E2" s="3" t="n"/>
+      <c r="F2" s="3" t="n"/>
+      <c r="G2" s="3" t="inlineStr">
         <is>
           <t>2026-04-20</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="n">
+      <c r="A3" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="3" t="inlineStr"/>
-      <c r="C3" s="3" t="inlineStr"/>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="B3" s="5" t="n"/>
+      <c r="C3" s="5" t="n"/>
+      <c r="D3" s="5" t="inlineStr">
         <is>
           <t>GCNA5EMJNXZPO57ARVJYQ5SN2DYYPD6ZCCENQ5AQTMVNKN77RDIPMI3A</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr"/>
-      <c r="F3" s="3" t="inlineStr"/>
-      <c r="G3" s="3" t="inlineStr">
+      <c r="E3" s="5" t="n"/>
+      <c r="F3" s="5" t="n"/>
+      <c r="G3" s="5" t="inlineStr">
         <is>
           <t>2026-04-20</t>
         </is>
@@ -559,35 +608,35 @@
       <c r="A4" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="2" t="inlineStr"/>
-      <c r="C4" s="2" t="inlineStr"/>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="B4" s="3" t="n"/>
+      <c r="C4" s="3" t="n"/>
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t>GALDPLQ62RAX3V7RJE73D3C2F4SKHGCJ3MIYJ4MLU2EAIUXBDSUVS7SA</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr"/>
-      <c r="F4" s="2" t="inlineStr"/>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="E4" s="3" t="n"/>
+      <c r="F4" s="3" t="n"/>
+      <c r="G4" s="3" t="inlineStr">
         <is>
           <t>2026-04-20</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="n">
+      <c r="A5" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="3" t="inlineStr"/>
-      <c r="C5" s="3" t="inlineStr"/>
-      <c r="D5" s="3" t="inlineStr">
+      <c r="B5" s="5" t="n"/>
+      <c r="C5" s="5" t="n"/>
+      <c r="D5" s="5" t="inlineStr">
         <is>
           <t>GDBOBVGP6HNLL66IOTSR6COGSZYRTSRDXBUD2CDDN3C5XGUT23TQ54J2</t>
         </is>
       </c>
-      <c r="E5" s="3" t="inlineStr"/>
-      <c r="F5" s="3" t="inlineStr"/>
-      <c r="G5" s="3" t="inlineStr">
+      <c r="E5" s="5" t="n"/>
+      <c r="F5" s="5" t="n"/>
+      <c r="G5" s="5" t="inlineStr">
         <is>
           <t>2026-04-20</t>
         </is>
@@ -597,35 +646,35 @@
       <c r="A6" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="2" t="inlineStr"/>
-      <c r="C6" s="2" t="inlineStr"/>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="B6" s="3" t="n"/>
+      <c r="C6" s="3" t="n"/>
+      <c r="D6" s="3" t="inlineStr">
         <is>
           <t>GAJXYRRBECPQVCOCCLBCCZ2KGGNEHL32TLJRT2JWLNVE4HJ35OAKAPH2</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr"/>
-      <c r="F6" s="2" t="inlineStr"/>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="E6" s="3" t="n"/>
+      <c r="F6" s="3" t="n"/>
+      <c r="G6" s="3" t="inlineStr">
         <is>
           <t>2026-04-20</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="n">
+      <c r="A7" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="3" t="inlineStr"/>
-      <c r="C7" s="3" t="inlineStr"/>
-      <c r="D7" s="3" t="inlineStr">
+      <c r="B7" s="5" t="n"/>
+      <c r="C7" s="5" t="n"/>
+      <c r="D7" s="5" t="inlineStr">
         <is>
           <t>GD72JZQAJPGLSLND6GPTSZ64PWMVY3JP5QKQJ32RW2GJCSVOSBPNX2EF</t>
         </is>
       </c>
-      <c r="E7" s="3" t="inlineStr"/>
-      <c r="F7" s="3" t="inlineStr"/>
-      <c r="G7" s="3" t="inlineStr">
+      <c r="E7" s="5" t="n"/>
+      <c r="F7" s="5" t="n"/>
+      <c r="G7" s="5" t="inlineStr">
         <is>
           <t>2026-04-20</t>
         </is>
@@ -635,34 +684,244 @@
       <c r="A8" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="2" t="inlineStr"/>
-      <c r="C8" s="2" t="inlineStr"/>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="B8" s="3" t="n"/>
+      <c r="C8" s="3" t="n"/>
+      <c r="D8" s="3" t="inlineStr">
         <is>
           <t>GDYAPFZH5R6EKEQKJ3TKLQPZQASNXSN5IYDPTQ7MBRLZGE5ABGYGK7M</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr"/>
-      <c r="F8" s="2" t="inlineStr"/>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="E8" s="3" t="n"/>
+      <c r="F8" s="3" t="n"/>
+      <c r="G8" s="3" t="inlineStr">
         <is>
           <t>2026-04-20</t>
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" s="6" t="n"/>
+      <c r="B9" s="6" t="n"/>
+      <c r="C9" s="6" t="n"/>
+      <c r="D9" s="6" t="n"/>
+      <c r="E9" s="6" t="n"/>
+      <c r="F9" s="6" t="n"/>
+      <c r="G9" s="6" t="n"/>
+    </row>
     <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>Note:</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="inlineStr">
-        <is>
-          <t>Rows 8–30+ will be populated as users submit the Google Form.</t>
+      <c r="A10" s="6" t="n"/>
+      <c r="B10" s="6" t="n"/>
+      <c r="C10" s="6" t="n"/>
+      <c r="D10" s="6" t="n"/>
+      <c r="E10" s="6" t="n"/>
+      <c r="F10" s="6" t="n"/>
+      <c r="G10" s="6" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="n"/>
+      <c r="B11" s="6" t="n"/>
+      <c r="C11" s="6" t="n"/>
+      <c r="D11" s="6" t="n"/>
+      <c r="E11" s="6" t="n"/>
+      <c r="F11" s="6" t="n"/>
+      <c r="G11" s="6" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="n"/>
+      <c r="B12" s="6" t="n"/>
+      <c r="C12" s="6" t="n"/>
+      <c r="D12" s="6" t="n"/>
+      <c r="E12" s="6" t="n"/>
+      <c r="F12" s="6" t="n"/>
+      <c r="G12" s="6" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="n"/>
+      <c r="B13" s="6" t="n"/>
+      <c r="C13" s="6" t="n"/>
+      <c r="D13" s="6" t="n"/>
+      <c r="E13" s="6" t="n"/>
+      <c r="F13" s="6" t="n"/>
+      <c r="G13" s="6" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="n"/>
+      <c r="B14" s="6" t="n"/>
+      <c r="C14" s="6" t="n"/>
+      <c r="D14" s="6" t="n"/>
+      <c r="E14" s="6" t="n"/>
+      <c r="F14" s="6" t="n"/>
+      <c r="G14" s="6" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="n"/>
+      <c r="B15" s="6" t="n"/>
+      <c r="C15" s="6" t="n"/>
+      <c r="D15" s="6" t="n"/>
+      <c r="E15" s="6" t="n"/>
+      <c r="F15" s="6" t="n"/>
+      <c r="G15" s="6" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="n"/>
+      <c r="B16" s="6" t="n"/>
+      <c r="C16" s="6" t="n"/>
+      <c r="D16" s="6" t="n"/>
+      <c r="E16" s="6" t="n"/>
+      <c r="F16" s="6" t="n"/>
+      <c r="G16" s="6" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="n"/>
+      <c r="B17" s="6" t="n"/>
+      <c r="C17" s="6" t="n"/>
+      <c r="D17" s="6" t="n"/>
+      <c r="E17" s="6" t="n"/>
+      <c r="F17" s="6" t="n"/>
+      <c r="G17" s="6" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="n"/>
+      <c r="B18" s="6" t="n"/>
+      <c r="C18" s="6" t="n"/>
+      <c r="D18" s="6" t="n"/>
+      <c r="E18" s="6" t="n"/>
+      <c r="F18" s="6" t="n"/>
+      <c r="G18" s="6" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="n"/>
+      <c r="B19" s="6" t="n"/>
+      <c r="C19" s="6" t="n"/>
+      <c r="D19" s="6" t="n"/>
+      <c r="E19" s="6" t="n"/>
+      <c r="F19" s="6" t="n"/>
+      <c r="G19" s="6" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="n"/>
+      <c r="B20" s="6" t="n"/>
+      <c r="C20" s="6" t="n"/>
+      <c r="D20" s="6" t="n"/>
+      <c r="E20" s="6" t="n"/>
+      <c r="F20" s="6" t="n"/>
+      <c r="G20" s="6" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="n"/>
+      <c r="B21" s="6" t="n"/>
+      <c r="C21" s="6" t="n"/>
+      <c r="D21" s="6" t="n"/>
+      <c r="E21" s="6" t="n"/>
+      <c r="F21" s="6" t="n"/>
+      <c r="G21" s="6" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="n"/>
+      <c r="B22" s="6" t="n"/>
+      <c r="C22" s="6" t="n"/>
+      <c r="D22" s="6" t="n"/>
+      <c r="E22" s="6" t="n"/>
+      <c r="F22" s="6" t="n"/>
+      <c r="G22" s="6" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="6" t="n"/>
+      <c r="B23" s="6" t="n"/>
+      <c r="C23" s="6" t="n"/>
+      <c r="D23" s="6" t="n"/>
+      <c r="E23" s="6" t="n"/>
+      <c r="F23" s="6" t="n"/>
+      <c r="G23" s="6" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="6" t="n"/>
+      <c r="B24" s="6" t="n"/>
+      <c r="C24" s="6" t="n"/>
+      <c r="D24" s="6" t="n"/>
+      <c r="E24" s="6" t="n"/>
+      <c r="F24" s="6" t="n"/>
+      <c r="G24" s="6" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="n"/>
+      <c r="B25" s="6" t="n"/>
+      <c r="C25" s="6" t="n"/>
+      <c r="D25" s="6" t="n"/>
+      <c r="E25" s="6" t="n"/>
+      <c r="F25" s="6" t="n"/>
+      <c r="G25" s="6" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="6" t="n"/>
+      <c r="B26" s="6" t="n"/>
+      <c r="C26" s="6" t="n"/>
+      <c r="D26" s="6" t="n"/>
+      <c r="E26" s="6" t="n"/>
+      <c r="F26" s="6" t="n"/>
+      <c r="G26" s="6" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="6" t="n"/>
+      <c r="B27" s="6" t="n"/>
+      <c r="C27" s="6" t="n"/>
+      <c r="D27" s="6" t="n"/>
+      <c r="E27" s="6" t="n"/>
+      <c r="F27" s="6" t="n"/>
+      <c r="G27" s="6" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="6" t="n"/>
+      <c r="B28" s="6" t="n"/>
+      <c r="C28" s="6" t="n"/>
+      <c r="D28" s="6" t="n"/>
+      <c r="E28" s="6" t="n"/>
+      <c r="F28" s="6" t="n"/>
+      <c r="G28" s="6" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="6" t="n"/>
+      <c r="B29" s="6" t="n"/>
+      <c r="C29" s="6" t="n"/>
+      <c r="D29" s="6" t="n"/>
+      <c r="E29" s="6" t="n"/>
+      <c r="F29" s="6" t="n"/>
+      <c r="G29" s="6" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="6" t="n"/>
+      <c r="B30" s="6" t="n"/>
+      <c r="C30" s="6" t="n"/>
+      <c r="D30" s="6" t="n"/>
+      <c r="E30" s="6" t="n"/>
+      <c r="F30" s="6" t="n"/>
+      <c r="G30" s="6" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="6" t="n"/>
+      <c r="B31" s="6" t="n"/>
+      <c r="C31" s="6" t="n"/>
+      <c r="D31" s="6" t="n"/>
+      <c r="E31" s="6" t="n"/>
+      <c r="F31" s="6" t="n"/>
+      <c r="G31" s="6" t="n"/>
+    </row>
+    <row r="32" ht="30" customHeight="1">
+      <c r="A32" s="7" t="inlineStr">
+        <is>
+          <t>ℹ Note</t>
+        </is>
+      </c>
+      <c r="B32" s="8" t="inlineStr">
+        <is>
+          <t>Rows 8–30+ are populated automatically when users submit the Google Form (https://forms.gle/stellarautopay). This file is re-exported from Google Sheets after each batch of new submissions.</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B32:G32"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -673,106 +932,298 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:B28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="35" customWidth="1" min="1" max="1"/>
-    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="38" customWidth="1" min="1" max="1"/>
+    <col width="70" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Metric</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Value</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="6" t="inlineStr">
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="9" t="inlineStr">
+        <is>
+          <t>📊  Response Statistics</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1">
+      <c r="A2" s="10" t="inlineStr">
         <is>
           <t>Total Responses Collected</t>
         </is>
       </c>
-      <c r="B2" s="6" t="n">
+      <c r="B2" s="11" t="n">
         <v>7</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="6" t="inlineStr">
+    <row r="3" ht="18" customHeight="1">
+      <c r="A3" s="10" t="inlineStr">
         <is>
           <t>Target Responses</t>
         </is>
       </c>
-      <c r="B3" s="6" t="n">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="6" t="inlineStr">
+      <c r="B3" s="12" t="inlineStr">
+        <is>
+          <t>30+</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="18" customHeight="1">
+      <c r="A4" s="10" t="inlineStr">
         <is>
           <t>Average Product Rating</t>
         </is>
       </c>
-      <c r="B4" s="6" t="inlineStr">
-        <is>
-          <t>Pending responses</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="6" t="inlineStr">
-        <is>
-          <t>Google Form Link</t>
-        </is>
-      </c>
-      <c r="B5" s="6" t="inlineStr">
+      <c r="B4" s="12" t="inlineStr">
+        <is>
+          <t>Pending — form responses needed</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="18" customHeight="1">
+      <c r="A5" s="10" t="inlineStr">
+        <is>
+          <t>Highest Rating Received</t>
+        </is>
+      </c>
+      <c r="B5" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="18" customHeight="1">
+      <c r="A6" s="10" t="inlineStr">
+        <is>
+          <t>Lowest Rating Received</t>
+        </is>
+      </c>
+      <c r="B6" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="18" customHeight="1">
+      <c r="A7" s="10" t="inlineStr">
+        <is>
+          <t>Last Updated</t>
+        </is>
+      </c>
+      <c r="B7" s="12" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="22" customHeight="1">
+      <c r="A9" s="9" t="inlineStr">
+        <is>
+          <t>🔗  Links &amp; References</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="18" customHeight="1">
+      <c r="A10" s="10" t="inlineStr">
+        <is>
+          <t>Google Form (submit feedback)</t>
+        </is>
+      </c>
+      <c r="B10" s="12" t="inlineStr">
         <is>
           <t>https://docs.google.com/forms/d/e/1FAIpQLSfp4qWFnQUWYiruEyvELlv1RJkK7_Q7UtrEXu4Ze-QmYMtb8A/viewform</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="6" t="inlineStr">
-        <is>
-          <t>Contract Address</t>
-        </is>
-      </c>
-      <c r="B6" s="6" t="inlineStr">
+    <row r="11" ht="18" customHeight="1">
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>Form Analytics Dashboard</t>
+        </is>
+      </c>
+      <c r="B11" s="12" t="inlineStr">
+        <is>
+          <t>https://docs.google.com/forms/d/e/1FAIpQLSfp4qWFnQUWYiruEyvELlv1RJkK7_Q7UtrEXu4Ze-QmYMtb8A/viewanalytics</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="18" customHeight="1">
+      <c r="A12" s="10" t="inlineStr">
+        <is>
+          <t>GitHub Repository</t>
+        </is>
+      </c>
+      <c r="B12" s="12" t="inlineStr">
+        <is>
+          <t>https://github.com/murat48/stellarautopay</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="18" customHeight="1">
+      <c r="A13" s="10" t="inlineStr">
+        <is>
+          <t>Smart Contract (Testnet)</t>
+        </is>
+      </c>
+      <c r="B13" s="12" t="inlineStr">
         <is>
           <t>CC3EMSSEYBKKMELWHKTQV422U2RJJ5FIN5CKBMJF2RPPUHSIGGKMMYUL</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="6" t="inlineStr">
+    <row r="14" ht="18" customHeight="1">
+      <c r="A14" s="10" t="inlineStr">
+        <is>
+          <t>Live Demo</t>
+        </is>
+      </c>
+      <c r="B14" s="12" t="inlineStr">
+        <is>
+          <t>https://stellarautopay.vercel.app</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="18" customHeight="1">
+      <c r="A15" s="10" t="inlineStr">
         <is>
           <t>Network</t>
         </is>
       </c>
-      <c r="B7" s="6" t="inlineStr">
+      <c r="B15" s="12" t="inlineStr">
         <is>
           <t>Stellar Testnet</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="6" t="inlineStr">
-        <is>
-          <t>Last Updated</t>
-        </is>
-      </c>
-      <c r="B8" s="6" t="inlineStr">
-        <is>
-          <t>2026-04-22</t>
+    <row r="17" ht="22" customHeight="1">
+      <c r="A17" s="9" t="inlineStr">
+        <is>
+          <t>⚙️  Data Collection Process</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="18" customHeight="1">
+      <c r="A18" s="10" t="inlineStr">
+        <is>
+          <t>Step 1</t>
+        </is>
+      </c>
+      <c r="B18" s="12" t="inlineStr">
+        <is>
+          <t>User fills Google Form → data flows automatically to Google Sheets</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="18" customHeight="1">
+      <c r="A19" s="10" t="inlineStr">
+        <is>
+          <t>Step 2</t>
+        </is>
+      </c>
+      <c r="B19" s="12" t="inlineStr">
+        <is>
+          <t>Maintainer exports Google Sheets → File → Download → .xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="18" customHeight="1">
+      <c r="A20" s="10" t="inlineStr">
+        <is>
+          <t>Step 3</t>
+        </is>
+      </c>
+      <c r="B20" s="12" t="inlineStr">
+        <is>
+          <t>Replace docs/user-feedback.xlsx in repository and commit</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="18" customHeight="1">
+      <c r="A21" s="10" t="inlineStr">
+        <is>
+          <t>Step 4</t>
+        </is>
+      </c>
+      <c r="B21" s="12" t="inlineStr">
+        <is>
+          <t>README table (rows 8–30+) is updated to reflect new wallet addresses</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="22" customHeight="1">
+      <c r="A23" s="9" t="inlineStr">
+        <is>
+          <t>📋  Google Form Fields</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="18" customHeight="1">
+      <c r="A24" s="10" t="inlineStr">
+        <is>
+          <t>Field 1</t>
+        </is>
+      </c>
+      <c r="B24" s="12" t="inlineStr">
+        <is>
+          <t>Full Name (Short answer — text)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="18" customHeight="1">
+      <c r="A25" s="10" t="inlineStr">
+        <is>
+          <t>Field 2</t>
+        </is>
+      </c>
+      <c r="B25" s="12" t="inlineStr">
+        <is>
+          <t>Email Address (Short answer — email validation)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="18" customHeight="1">
+      <c r="A26" s="10" t="inlineStr">
+        <is>
+          <t>Field 3</t>
+        </is>
+      </c>
+      <c r="B26" s="12" t="inlineStr">
+        <is>
+          <t>Stellar Testnet Wallet Address (Short answer — starts with G)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="18" customHeight="1">
+      <c r="A27" s="10" t="inlineStr">
+        <is>
+          <t>Field 4</t>
+        </is>
+      </c>
+      <c r="B27" s="12" t="inlineStr">
+        <is>
+          <t>Product Rating (Linear scale 1–5 ★)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="18" customHeight="1">
+      <c r="A28" s="10" t="inlineStr">
+        <is>
+          <t>Field 5</t>
+        </is>
+      </c>
+      <c r="B28" s="12" t="inlineStr">
+        <is>
+          <t>Comments / Suggestions (Paragraph — optional)</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="A9:B9"/>
+    <mergeCell ref="A23:B23"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="A17:B17"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>